<commit_message>
mise à jour des pages générées de l'ig
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-fr-core-location.xlsx
+++ b/docs/StructureDefinition-fr-core-location.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-02T16:31:57+01:00</t>
+    <t>2025-11-02T18:22:16+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G9" t="s" s="2">
         <v>78</v>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s" s="2">
         <v>85</v>

</xml_diff>